<commit_message>
Add IC Memo tabs to all Model files
- Added 'IC Memo' sheet to Model_1 through Model_5
- Content extracted from IC_Memo_*.docx files
- Sheets verified: [Model, IC Memo]
- Regenerated deliverables ZIP
</commit_message>
<xml_diff>
--- a/deliverables/deliverables-20260120-0030/Model_1_CCGT.xlsx
+++ b/deliverables/deliverables-20260120-0030/Model_1_CCGT.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IC Memo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,6 +53,25 @@
     <font>
       <b val="1"/>
       <color rgb="000000FF"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -104,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -137,6 +157,18 @@
     <xf numFmtId="166" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -622,7 +654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N159"/>
+  <dimension ref="A1:N135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -911,8 +943,6 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -1013,7 +1043,6 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
@@ -1114,7 +1143,6 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
@@ -1215,7 +1243,6 @@
         <v>0.025</v>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
@@ -1276,7 +1303,6 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
@@ -1417,7 +1443,6 @@
         <v>1.1</v>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
@@ -1498,8 +1523,6 @@
         <v>15</v>
       </c>
     </row>
-    <row r="50"/>
-    <row r="51"/>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
@@ -1625,8 +1648,6 @@
         <v/>
       </c>
     </row>
-    <row r="58"/>
-    <row r="59"/>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
@@ -1818,7 +1839,6 @@
         <v/>
       </c>
     </row>
-    <row r="64"/>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
@@ -1986,7 +2006,6 @@
         <v/>
       </c>
     </row>
-    <row r="68"/>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
@@ -2211,7 +2230,6 @@
         <v/>
       </c>
     </row>
-    <row r="73"/>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
@@ -2269,8 +2287,6 @@
         <v/>
       </c>
     </row>
-    <row r="75"/>
-    <row r="76"/>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
@@ -2462,8 +2478,6 @@
         <v/>
       </c>
     </row>
-    <row r="81"/>
-    <row r="82"/>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
@@ -3054,7 +3068,6 @@
         <v/>
       </c>
     </row>
-    <row r="94"/>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
@@ -3315,8 +3328,6 @@
         <v/>
       </c>
     </row>
-    <row r="100"/>
-    <row r="101"/>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
@@ -3504,8 +3515,6 @@
         <v/>
       </c>
     </row>
-    <row r="106"/>
-    <row r="107"/>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
@@ -3603,7 +3612,6 @@
         <v/>
       </c>
     </row>
-    <row r="114"/>
     <row r="115">
       <c r="A115" s="23" t="inlineStr">
         <is>
@@ -3681,8 +3689,6 @@
         <v/>
       </c>
     </row>
-    <row r="120"/>
-    <row r="121"/>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
@@ -3787,7 +3793,6 @@
         <v/>
       </c>
     </row>
-    <row r="127"/>
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
@@ -3907,7 +3912,6 @@
         <v/>
       </c>
     </row>
-    <row r="132"/>
     <row r="133">
       <c r="A133" s="23" t="inlineStr">
         <is>
@@ -3995,32 +3999,661 @@
         <v/>
       </c>
     </row>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A92"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>PROJECT SPARTAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="29" t="inlineStr">
+        <is>
+          <t>INVESTMENT COMMITTEE MEMORANDUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>365 MW Combined Cycle Gas Turbine – PJM West</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>RECOMMENDATION: Proceed to final bid at $520mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>KEY METRICS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>INVESTMENT THESIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>• Strategic PJM West location with dual revenue streams (energy + capacity) provides diversified cash flow profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>• Efficient 7,000 Btu/kWh heat rate positions asset competitively on dispatch stack, ensuring consistent energy margins</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="28" t="inlineStr">
+        <is>
+          <t>• Recent PJM capacity auction results support sustained capacity revenue outlook through the hold period</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>• Clear exit path to strategic buyers (utilities seeking gas generation) and infrastructure yield vehicles</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>KEY RISKS &amp; MITIGANTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>FINANCING STRUCTURE RATIONALE</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>Structure: 7-year term loan with 75% cash sweep and 6-month DSRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="28" t="inlineStr">
+        <is>
+          <t>Rationale:</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
+        <is>
+          <t>• Cash sweep structure appropriate for merchant asset with variable CFADS – accelerates paydown in strong years</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>• 45% leverage balances return enhancement with covenant headroom for commodity cycles</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>• 6-month DSRA provides liquidity buffer, sizing is market standard for merchant power</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>• Lock-up DSCR at 1.10x protects lenders while allowing distributions in base case</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="inlineStr">
+        <is>
+          <t>ANTICIPATED IC Q&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="29" t="inlineStr">
+        <is>
+          <t>VALUATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="29" t="inlineStr">
+        <is>
+          <t>Q: How did you arrive at 7.8x entry multiple?</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="28" t="inlineStr">
+        <is>
+          <t>A: Based on recent PJM CCGT transactions ranging 7.0-8.5x, adjusted down for merchant exposure vs contracted comps. Premium to replacement cost reflects strategic location and grid constraints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="inlineStr">
+        <is>
+          <t>Q: What's the exit buyer universe?</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="28" t="inlineStr">
+        <is>
+          <t>A: Primary: Utilities seeking gas generation for reliability (AES, NRG, Vistra). Secondary: Infrastructure funds (KKR, Brookfield, GIP) seeking yield with upside. Tertiary: IPPs for portfolio buildout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="29" t="inlineStr">
+        <is>
+          <t>Q: Why 7.0x exit multiple vs 7.8x entry?</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="28" t="inlineStr">
+        <is>
+          <t>A: Conservative assumption reflects shorter remaining life at exit. Sensitivity shows 0.5x multiple change = 200bps IRR impact.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="29" t="inlineStr">
+        <is>
+          <t>FINANCING</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="29" t="inlineStr">
+        <is>
+          <t>Q: Why sweep instead of sculpt?</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="28" t="inlineStr">
+        <is>
+          <t>A: Merchant CFADS volatility makes sculpting impractical – you'd need to re-sculpt every year. Sweep naturally adjusts paydown to actual cash flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="inlineStr">
+        <is>
+          <t>Q: How did you size the DSRA?</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
+          <t>A: 6-month debt service is market standard for merchant power. Provides 6 months of runway if spark spreads compress or outage occurs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>Q: What happens if DSCR drops below 1.10x?</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="28" t="inlineStr">
+        <is>
+          <t>A: Distributions locked up – all excess cash goes to debt paydown. Likely scenario: temporary commodity dislocation. Recovery expected within 1-2 years.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="29" t="inlineStr">
+        <is>
+          <t>RETURNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="30" t="inlineStr">
+        <is>
+          <t>Q: Walk me through the IRR bridge from unlevered to levered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="28" t="inlineStr">
+        <is>
+          <t>A: Unlevered 12.1% + leverage benefit (cheaper debt vs equity cost) ≈ +7% – financing costs (interest, fees) ≈ -0.6% = Levered 18.5%. Leverage adds ~6.5% to returns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="30" t="inlineStr">
+        <is>
+          <t>Q: Why is MOIC 2.15x lower than I'd expect for 18.5% IRR?</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="28" t="inlineStr">
+        <is>
+          <t>A: 7-year hold period. MOIC = cash-on-cash regardless of timing. 18.5% IRR over 7 years compounds to 2.15x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="29" t="inlineStr">
+        <is>
+          <t>Q: What's the downside scenario?</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="28" t="inlineStr">
+        <is>
+          <t>A: Gas +25%, power flat = squeezed spark spreads. IRR drops to 14.2%, still above hurdle. DSCR 1.28x maintains covenant compliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="29" t="inlineStr">
+        <is>
+          <t>MARKET</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="29" t="inlineStr">
+        <is>
+          <t>Q: What happens if PJM capacity prices collapse?</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="28" t="inlineStr">
+        <is>
+          <t>A: Downside scenario assumes 20% capacity price decline. Still economic due to energy revenue diversification. Extreme downside: asset becomes peaker-like, relies on scarcity pricing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="30" t="inlineStr">
+        <is>
+          <t>Q: How does carbon regulation affect the investment?</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="28" t="inlineStr">
+        <is>
+          <t>A: Gas is bridge fuel – CCGTs run when renewables can't. Carbon cost would increase power prices, potentially improving spark spreads. Natural gas is 50% lower emissions than coal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="29" t="inlineStr">
+        <is>
+          <t>OPERATIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="29" t="inlineStr">
+        <is>
+          <t>Q: What are the key operational risks?</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="28" t="inlineStr">
+        <is>
+          <t>A: Equipment failure (mitigated by LTSA), fuel supply disruption (mitigated by pipeline redundancy), grid curtailment (mitigated by must-run status).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="29" t="inlineStr">
+        <is>
+          <t>Q: What value creation levers exist?</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="28" t="inlineStr">
+        <is>
+          <t>A: 1) Heat rate improvement project (+$2mm EBITDA), 2) Ancillary services expansion, 3) Capacity factor optimization through better dispatch strategy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="28" t="inlineStr">
+        <is>
+          <t>────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="29" t="inlineStr">
+        <is>
+          <t>DILIGENCE PLAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="29" t="inlineStr">
+        <is>
+          <t>Technical:</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="28" t="inlineStr">
+        <is>
+          <t>☐ Independent engineer report (Wood Mackenzie)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="28" t="inlineStr">
+        <is>
+          <t>☐ Equipment condition assessment – turbine hours remaining</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="28" t="inlineStr">
+        <is>
+          <t>☐ Environmental compliance review – air permits, water discharge</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="28" t="inlineStr">
+        <is>
+          <t>☐ Grid interconnection study – transmission constraints</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="29" t="inlineStr">
+        <is>
+          <t>Commercial:</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="28" t="inlineStr">
+        <is>
+          <t>☐ PPA/hedging contract review</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="28" t="inlineStr">
+        <is>
+          <t>☐ Market study validation (ERCOT/PJM consultant)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="28" t="inlineStr">
+        <is>
+          <t>☐ Fuel supply and transportation agreements</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="28" t="inlineStr">
+        <is>
+          <t>☐ Counterparty credit analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="29" t="inlineStr">
+        <is>
+          <t>Legal:</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="28" t="inlineStr">
+        <is>
+          <t>☐ Title and land rights review</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="28" t="inlineStr">
+        <is>
+          <t>☐ Permitting status and renewal timeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="28" t="inlineStr">
+        <is>
+          <t>☐ Environmental liability assessment</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="28" t="inlineStr">
+        <is>
+          <t>☐ Regulatory status and rate case history</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="29" t="inlineStr">
+        <is>
+          <t>Financial:</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="28" t="inlineStr">
+        <is>
+          <t>☐ Quality of earnings (trailing 3-year analysis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="28" t="inlineStr">
+        <is>
+          <t>☐ Working capital normalization</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="28" t="inlineStr">
+        <is>
+          <t>☐ Tax structure optimization</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="28" t="inlineStr">
+        <is>
+          <t>☐ Insurance adequacy review</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="28" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="31" t="inlineStr">
+        <is>
+          <t>Metric | Base Case | Downside | Upside</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="31" t="inlineStr">
+        <is>
+          <t>Entry EV | $520mm | - | -</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="31" t="inlineStr">
+        <is>
+          <t>Entry Multiple | 7.8x Y1 EBITDA | - | -</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="31" t="inlineStr">
+        <is>
+          <t>Leverage | 45% | - | -</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="31" t="inlineStr">
+        <is>
+          <t>Levered IRR | 18.5% | 14.2% | 22.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="31" t="inlineStr">
+        <is>
+          <t>MOIC | 2.15x | 1.85x | 2.45x</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="31" t="inlineStr">
+        <is>
+          <t>Min DSCR | 1.42x | 1.28x | 1.58x</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="31" t="inlineStr">
+        <is>
+          <t>Unlevered IRR | 12.1% | - | -</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="28" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="31" t="inlineStr">
+        <is>
+          <t>Risk | Probability | Mitigant</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="31" t="inlineStr">
+        <is>
+          <t>Gas price volatility | Medium | Partial hedge program (50% Y1-Y3); efficient heat rate provides margin cushion</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="31" t="inlineStr">
+        <is>
+          <t>Capacity price decline | Medium | PJM capacity construct provides 3-year forward visibility; locked through Y3</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="31" t="inlineStr">
+        <is>
+          <t>Forced outage risk | Low | Comprehensive LTSA with OEM; historical 95% availability; 6-month DSRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="31" t="inlineStr">
+        <is>
+          <t>Environmental regulation | Medium | No pending EPA action on unit; brownfield expansion rights provide optionality</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>